<commit_message>
v.2.4.2: calcula 9 novos indicadores dos bancos consolidados, exclui ipynb e atualiza bases
</commit_message>
<xml_diff>
--- a/data/Consolidação 03 - script_03_rotas.xlsx
+++ b/data/Consolidação 03 - script_03_rotas.xlsx
@@ -1,26 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5be72e984ffd378f/Documentos/UFG/CECATE/PDDE_extracao_selects (1)/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_583147CBD34AAE2E137B2D11595ED87656CDB3F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="12645" yWindow="2235" windowWidth="2715" windowHeight="8565" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="consolidado" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
   <si>
     <t>estado</t>
   </si>
@@ -58,22 +52,37 @@
     <t>sem_da_ponterustica</t>
   </si>
   <si>
-    <t>rotas_rodoviarias</t>
-  </si>
-  <si>
-    <t>rotas_aquaviarias</t>
-  </si>
-  <si>
-    <t>rotas_mistas</t>
-  </si>
-  <si>
-    <t>rotas_tipo_nao_identificado</t>
-  </si>
-  <si>
-    <t>rotas_geoferenciadas</t>
-  </si>
-  <si>
-    <t>rotas_nao_georeferenciadas</t>
+    <t>rodoviaria</t>
+  </si>
+  <si>
+    <t>aquaviaria</t>
+  </si>
+  <si>
+    <t>mista</t>
+  </si>
+  <si>
+    <t>tipo_nao_informado</t>
+  </si>
+  <si>
+    <t>turno_matutino</t>
+  </si>
+  <si>
+    <t>turno_vespertino</t>
+  </si>
+  <si>
+    <t>turno_noturno</t>
+  </si>
+  <si>
+    <t>rota_ativa</t>
+  </si>
+  <si>
+    <t>rota_inativa</t>
+  </si>
+  <si>
+    <t>com_georreferenciamento</t>
+  </si>
+  <si>
+    <t>sem_georreferenciamento</t>
   </si>
   <si>
     <t>Acre</t>
@@ -155,13 +164,16 @@
   </si>
   <si>
     <t>Tocantins</t>
+  </si>
+  <si>
+    <t>Brasil</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -172,8 +184,10 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -222,14 +236,6 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -517,11 +523,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R28"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:W29"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -576,10 +582,25 @@
       <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:23">
       <c r="A2" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="B2">
         <v>128</v>
@@ -627,15 +648,30 @@
         <v>0</v>
       </c>
       <c r="Q2">
+        <v>120</v>
+      </c>
+      <c r="R2">
+        <v>59</v>
+      </c>
+      <c r="S2">
+        <v>5</v>
+      </c>
+      <c r="T2">
+        <v>128</v>
+      </c>
+      <c r="U2">
+        <v>0</v>
+      </c>
+      <c r="V2">
         <v>24</v>
       </c>
-      <c r="R2">
+      <c r="W2">
         <v>104</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:23">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="B3">
         <v>1345</v>
@@ -683,15 +719,30 @@
         <v>0</v>
       </c>
       <c r="Q3">
+        <v>876</v>
+      </c>
+      <c r="R3">
+        <v>861</v>
+      </c>
+      <c r="S3">
+        <v>277</v>
+      </c>
+      <c r="T3">
+        <v>1344</v>
+      </c>
+      <c r="U3">
+        <v>1</v>
+      </c>
+      <c r="V3">
         <v>762</v>
       </c>
-      <c r="R3">
+      <c r="W3">
         <v>583</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:23">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="B4">
         <v>47</v>
@@ -739,15 +790,30 @@
         <v>0</v>
       </c>
       <c r="Q4">
+        <v>46</v>
+      </c>
+      <c r="R4">
+        <v>45</v>
+      </c>
+      <c r="S4">
+        <v>3</v>
+      </c>
+      <c r="T4">
+        <v>47</v>
+      </c>
+      <c r="U4">
+        <v>0</v>
+      </c>
+      <c r="V4">
         <v>1</v>
       </c>
-      <c r="R4">
+      <c r="W4">
         <v>46</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:23">
       <c r="A5" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="B5">
         <v>332</v>
@@ -795,15 +861,30 @@
         <v>0</v>
       </c>
       <c r="Q5">
+        <v>235</v>
+      </c>
+      <c r="R5">
+        <v>175</v>
+      </c>
+      <c r="S5">
+        <v>39</v>
+      </c>
+      <c r="T5">
+        <v>332</v>
+      </c>
+      <c r="U5">
+        <v>0</v>
+      </c>
+      <c r="V5">
         <v>191</v>
       </c>
-      <c r="R5">
+      <c r="W5">
         <v>141</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:23">
       <c r="A6" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="B6">
         <v>10080</v>
@@ -851,15 +932,30 @@
         <v>0</v>
       </c>
       <c r="Q6">
+        <v>6935</v>
+      </c>
+      <c r="R6">
+        <v>5960</v>
+      </c>
+      <c r="S6">
+        <v>1861</v>
+      </c>
+      <c r="T6">
+        <v>9884</v>
+      </c>
+      <c r="U6">
+        <v>196</v>
+      </c>
+      <c r="V6">
         <v>3748</v>
       </c>
-      <c r="R6">
+      <c r="W6">
         <v>6332</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:23">
       <c r="A7" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B7">
         <v>4382</v>
@@ -907,15 +1003,30 @@
         <v>0</v>
       </c>
       <c r="Q7">
+        <v>3564</v>
+      </c>
+      <c r="R7">
+        <v>3392</v>
+      </c>
+      <c r="S7">
+        <v>272</v>
+      </c>
+      <c r="T7">
+        <v>4376</v>
+      </c>
+      <c r="U7">
+        <v>6</v>
+      </c>
+      <c r="V7">
         <v>586</v>
       </c>
-      <c r="R7">
+      <c r="W7">
         <v>3796</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:23">
       <c r="A8" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="B8">
         <v>5</v>
@@ -963,15 +1074,30 @@
         <v>0</v>
       </c>
       <c r="Q8">
+        <v>4</v>
+      </c>
+      <c r="R8">
+        <v>4</v>
+      </c>
+      <c r="S8">
+        <v>0</v>
+      </c>
+      <c r="T8">
+        <v>5</v>
+      </c>
+      <c r="U8">
+        <v>0</v>
+      </c>
+      <c r="V8">
         <v>3</v>
       </c>
-      <c r="R8">
+      <c r="W8">
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:23">
       <c r="A9" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="B9">
         <v>1971</v>
@@ -1019,15 +1145,30 @@
         <v>0</v>
       </c>
       <c r="Q9">
+        <v>1400</v>
+      </c>
+      <c r="R9">
+        <v>932</v>
+      </c>
+      <c r="S9">
+        <v>95</v>
+      </c>
+      <c r="T9">
+        <v>1971</v>
+      </c>
+      <c r="U9">
+        <v>0</v>
+      </c>
+      <c r="V9">
         <v>622</v>
       </c>
-      <c r="R9">
+      <c r="W9">
         <v>1349</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:23">
       <c r="A10" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="B10">
         <v>2491</v>
@@ -1075,15 +1216,30 @@
         <v>0</v>
       </c>
       <c r="Q10">
+        <v>1729</v>
+      </c>
+      <c r="R10">
+        <v>1543</v>
+      </c>
+      <c r="S10">
+        <v>230</v>
+      </c>
+      <c r="T10">
+        <v>2491</v>
+      </c>
+      <c r="U10">
+        <v>0</v>
+      </c>
+      <c r="V10">
         <v>887</v>
       </c>
-      <c r="R10">
+      <c r="W10">
         <v>1604</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:23">
       <c r="A11" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="B11">
         <v>1968</v>
@@ -1131,15 +1287,30 @@
         <v>0</v>
       </c>
       <c r="Q11">
+        <v>1388</v>
+      </c>
+      <c r="R11">
+        <v>1455</v>
+      </c>
+      <c r="S11">
+        <v>221</v>
+      </c>
+      <c r="T11">
+        <v>1967</v>
+      </c>
+      <c r="U11">
+        <v>1</v>
+      </c>
+      <c r="V11">
         <v>505</v>
       </c>
-      <c r="R11">
+      <c r="W11">
         <v>1463</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23">
       <c r="A12" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="B12">
         <v>2199</v>
@@ -1187,15 +1358,30 @@
         <v>0</v>
       </c>
       <c r="Q12">
+        <v>1410</v>
+      </c>
+      <c r="R12">
+        <v>1277</v>
+      </c>
+      <c r="S12">
+        <v>106</v>
+      </c>
+      <c r="T12">
+        <v>2199</v>
+      </c>
+      <c r="U12">
+        <v>0</v>
+      </c>
+      <c r="V12">
         <v>697</v>
       </c>
-      <c r="R12">
+      <c r="W12">
         <v>1502</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23">
       <c r="A13" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="B13">
         <v>1245</v>
@@ -1243,15 +1429,30 @@
         <v>0</v>
       </c>
       <c r="Q13">
+        <v>963</v>
+      </c>
+      <c r="R13">
+        <v>654</v>
+      </c>
+      <c r="S13">
+        <v>123</v>
+      </c>
+      <c r="T13">
+        <v>1245</v>
+      </c>
+      <c r="U13">
+        <v>0</v>
+      </c>
+      <c r="V13">
         <v>483</v>
       </c>
-      <c r="R13">
+      <c r="W13">
         <v>762</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23">
       <c r="A14" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="B14">
         <v>15679</v>
@@ -1299,15 +1500,30 @@
         <v>0</v>
       </c>
       <c r="Q14">
+        <v>11210</v>
+      </c>
+      <c r="R14">
+        <v>9115</v>
+      </c>
+      <c r="S14">
+        <v>1648</v>
+      </c>
+      <c r="T14">
+        <v>15664</v>
+      </c>
+      <c r="U14">
+        <v>15</v>
+      </c>
+      <c r="V14">
         <v>5855</v>
       </c>
-      <c r="R14">
+      <c r="W14">
         <v>9824</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:23">
       <c r="A15" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="B15">
         <v>6095</v>
@@ -1355,15 +1571,30 @@
         <v>0</v>
       </c>
       <c r="Q15">
+        <v>3858</v>
+      </c>
+      <c r="R15">
+        <v>3462</v>
+      </c>
+      <c r="S15">
+        <v>497</v>
+      </c>
+      <c r="T15">
+        <v>6093</v>
+      </c>
+      <c r="U15">
+        <v>2</v>
+      </c>
+      <c r="V15">
         <v>3893</v>
       </c>
-      <c r="R15">
+      <c r="W15">
         <v>2202</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:23">
       <c r="A16" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="B16">
         <v>1715</v>
@@ -1411,15 +1642,30 @@
         <v>0</v>
       </c>
       <c r="Q16">
+        <v>1180</v>
+      </c>
+      <c r="R16">
+        <v>1003</v>
+      </c>
+      <c r="S16">
+        <v>250</v>
+      </c>
+      <c r="T16">
+        <v>1713</v>
+      </c>
+      <c r="U16">
+        <v>2</v>
+      </c>
+      <c r="V16">
         <v>284</v>
       </c>
-      <c r="R16">
+      <c r="W16">
         <v>1431</v>
       </c>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:23">
       <c r="A17" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="B17">
         <v>3235</v>
@@ -1467,15 +1713,30 @@
         <v>0</v>
       </c>
       <c r="Q17">
+        <v>2212</v>
+      </c>
+      <c r="R17">
+        <v>2128</v>
+      </c>
+      <c r="S17">
+        <v>318</v>
+      </c>
+      <c r="T17">
+        <v>3234</v>
+      </c>
+      <c r="U17">
+        <v>1</v>
+      </c>
+      <c r="V17">
         <v>595</v>
       </c>
-      <c r="R17">
+      <c r="W17">
         <v>2640</v>
       </c>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:23">
       <c r="A18" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="B18">
         <v>6139</v>
@@ -1523,15 +1784,30 @@
         <v>0</v>
       </c>
       <c r="Q18">
+        <v>4083</v>
+      </c>
+      <c r="R18">
+        <v>3640</v>
+      </c>
+      <c r="S18">
+        <v>808</v>
+      </c>
+      <c r="T18">
+        <v>6139</v>
+      </c>
+      <c r="U18">
+        <v>0</v>
+      </c>
+      <c r="V18">
         <v>3036</v>
       </c>
-      <c r="R18">
+      <c r="W18">
         <v>3103</v>
       </c>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:23">
       <c r="A19" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="B19">
         <v>1928</v>
@@ -1579,15 +1855,30 @@
         <v>0</v>
       </c>
       <c r="Q19">
+        <v>1377</v>
+      </c>
+      <c r="R19">
+        <v>1397</v>
+      </c>
+      <c r="S19">
+        <v>120</v>
+      </c>
+      <c r="T19">
+        <v>1925</v>
+      </c>
+      <c r="U19">
+        <v>3</v>
+      </c>
+      <c r="V19">
         <v>694</v>
       </c>
-      <c r="R19">
+      <c r="W19">
         <v>1234</v>
       </c>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:23">
       <c r="A20" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="B20">
         <v>1188</v>
@@ -1635,15 +1926,30 @@
         <v>0</v>
       </c>
       <c r="Q20">
+        <v>779</v>
+      </c>
+      <c r="R20">
+        <v>702</v>
+      </c>
+      <c r="S20">
+        <v>252</v>
+      </c>
+      <c r="T20">
+        <v>1188</v>
+      </c>
+      <c r="U20">
+        <v>0</v>
+      </c>
+      <c r="V20">
         <v>385</v>
       </c>
-      <c r="R20">
+      <c r="W20">
         <v>803</v>
       </c>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:23">
       <c r="A21" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="B21">
         <v>6522</v>
@@ -1691,15 +1997,30 @@
         <v>0</v>
       </c>
       <c r="Q21">
+        <v>4679</v>
+      </c>
+      <c r="R21">
+        <v>4438</v>
+      </c>
+      <c r="S21">
+        <v>535</v>
+      </c>
+      <c r="T21">
+        <v>6505</v>
+      </c>
+      <c r="U21">
+        <v>17</v>
+      </c>
+      <c r="V21">
         <v>3068</v>
       </c>
-      <c r="R21">
+      <c r="W21">
         <v>3454</v>
       </c>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:23">
       <c r="A22" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="B22">
         <v>1078</v>
@@ -1747,15 +2068,30 @@
         <v>0</v>
       </c>
       <c r="Q22">
+        <v>883</v>
+      </c>
+      <c r="R22">
+        <v>792</v>
+      </c>
+      <c r="S22">
+        <v>59</v>
+      </c>
+      <c r="T22">
+        <v>1078</v>
+      </c>
+      <c r="U22">
+        <v>0</v>
+      </c>
+      <c r="V22">
         <v>321</v>
       </c>
-      <c r="R22">
+      <c r="W22">
         <v>757</v>
       </c>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:23">
       <c r="A23" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B23">
         <v>1362</v>
@@ -1803,15 +2139,30 @@
         <v>0</v>
       </c>
       <c r="Q23">
+        <v>743</v>
+      </c>
+      <c r="R23">
+        <v>750</v>
+      </c>
+      <c r="S23">
+        <v>24</v>
+      </c>
+      <c r="T23">
+        <v>1362</v>
+      </c>
+      <c r="U23">
+        <v>0</v>
+      </c>
+      <c r="V23">
         <v>500</v>
       </c>
-      <c r="R23">
+      <c r="W23">
         <v>862</v>
       </c>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:23">
       <c r="A24" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B24">
         <v>62</v>
@@ -1859,15 +2210,30 @@
         <v>0</v>
       </c>
       <c r="Q24">
+        <v>55</v>
+      </c>
+      <c r="R24">
+        <v>31</v>
+      </c>
+      <c r="S24">
+        <v>0</v>
+      </c>
+      <c r="T24">
+        <v>62</v>
+      </c>
+      <c r="U24">
+        <v>0</v>
+      </c>
+      <c r="V24">
         <v>26</v>
       </c>
-      <c r="R24">
+      <c r="W24">
         <v>36</v>
       </c>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:23">
       <c r="A25" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="B25">
         <v>2839</v>
@@ -1915,15 +2281,30 @@
         <v>0</v>
       </c>
       <c r="Q25">
+        <v>2099</v>
+      </c>
+      <c r="R25">
+        <v>2054</v>
+      </c>
+      <c r="S25">
+        <v>466</v>
+      </c>
+      <c r="T25">
+        <v>2834</v>
+      </c>
+      <c r="U25">
+        <v>5</v>
+      </c>
+      <c r="V25">
         <v>1462</v>
       </c>
-      <c r="R25">
+      <c r="W25">
         <v>1377</v>
       </c>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:23">
       <c r="A26" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B26">
         <v>574</v>
@@ -1971,15 +2352,30 @@
         <v>0</v>
       </c>
       <c r="Q26">
+        <v>405</v>
+      </c>
+      <c r="R26">
+        <v>392</v>
+      </c>
+      <c r="S26">
+        <v>95</v>
+      </c>
+      <c r="T26">
+        <v>574</v>
+      </c>
+      <c r="U26">
+        <v>0</v>
+      </c>
+      <c r="V26">
         <v>300</v>
       </c>
-      <c r="R26">
+      <c r="W26">
         <v>274</v>
       </c>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:23">
       <c r="A27" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B27">
         <v>6632</v>
@@ -2027,15 +2423,30 @@
         <v>0</v>
       </c>
       <c r="Q27">
+        <v>4298</v>
+      </c>
+      <c r="R27">
+        <v>4139</v>
+      </c>
+      <c r="S27">
+        <v>637</v>
+      </c>
+      <c r="T27">
+        <v>6631</v>
+      </c>
+      <c r="U27">
+        <v>1</v>
+      </c>
+      <c r="V27">
         <v>1801</v>
       </c>
-      <c r="R27">
+      <c r="W27">
         <v>4831</v>
       </c>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:23">
       <c r="A28" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B28">
         <v>1646</v>
@@ -2083,13 +2494,99 @@
         <v>0</v>
       </c>
       <c r="Q28">
+        <v>921</v>
+      </c>
+      <c r="R28">
+        <v>1078</v>
+      </c>
+      <c r="S28">
+        <v>175</v>
+      </c>
+      <c r="T28">
+        <v>1646</v>
+      </c>
+      <c r="U28">
+        <v>0</v>
+      </c>
+      <c r="V28">
         <v>897</v>
       </c>
-      <c r="R28">
+      <c r="W28">
         <v>749</v>
       </c>
     </row>
+    <row r="29" spans="1:23">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29">
+        <v>82887</v>
+      </c>
+      <c r="C29">
+        <v>6061</v>
+      </c>
+      <c r="D29">
+        <v>76826</v>
+      </c>
+      <c r="E29">
+        <v>7896</v>
+      </c>
+      <c r="F29">
+        <v>74991</v>
+      </c>
+      <c r="G29">
+        <v>2906</v>
+      </c>
+      <c r="H29">
+        <v>79981</v>
+      </c>
+      <c r="I29">
+        <v>9524</v>
+      </c>
+      <c r="J29">
+        <v>73363</v>
+      </c>
+      <c r="K29">
+        <v>5701</v>
+      </c>
+      <c r="L29">
+        <v>77186</v>
+      </c>
+      <c r="M29">
+        <v>76616</v>
+      </c>
+      <c r="N29">
+        <v>1693</v>
+      </c>
+      <c r="O29">
+        <v>4578</v>
+      </c>
+      <c r="P29">
+        <v>0</v>
+      </c>
+      <c r="Q29">
+        <v>57452</v>
+      </c>
+      <c r="R29">
+        <v>51478</v>
+      </c>
+      <c r="S29">
+        <v>9116</v>
+      </c>
+      <c r="T29">
+        <v>82637</v>
+      </c>
+      <c r="U29">
+        <v>250</v>
+      </c>
+      <c r="V29">
+        <v>31626</v>
+      </c>
+      <c r="W29">
+        <v>51261</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>